<commit_message>
Update Total Prompts to 55 and recalculate ratio to 10.91%
</commit_message>
<xml_diff>
--- a/ai_logs/Phuc_AI_AuditLog.xlsx
+++ b/ai_logs/Phuc_AI_AuditLog.xlsx
@@ -668,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" style="32" min="1" max="1"/>
@@ -764,7 +764,7 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11">
@@ -785,7 +785,7 @@
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>10.91%</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -1013,6 +1013,9 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Fix student name and ID in metadata
</commit_message>
<xml_diff>
--- a/ai_logs/Phuc_AI_AuditLog.xlsx
+++ b/ai_logs/Phuc_AI_AuditLog.xlsx
@@ -668,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" style="32" min="1" max="1"/>
@@ -703,7 +703,7 @@
       </c>
       <c r="C4" s="32" t="inlineStr">
         <is>
-          <t>[Enter your name]</t>
+          <t>Hoang Phuc</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="C5" s="32" t="inlineStr">
         <is>
-          <t>Lê Đỗ Hoàng Phúc</t>
+          <t>QE...</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>QE200057</t>
+          <t>CSD201</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="C7" s="32" t="inlineStr">
         <is>
-          <t>CSD201</t>
+          <t>Browser History</t>
         </is>
       </c>
     </row>
@@ -928,7 +928,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="18.75" customHeight="1" s="35">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -1013,9 +1012,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Rewrite logs to remove personal pronouns for a more professional tone
</commit_message>
<xml_diff>
--- a/ai_logs/Phuc_AI_AuditLog.xlsx
+++ b/ai_logs/Phuc_AI_AuditLog.xlsx
@@ -211,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -298,9 +298,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -668,7 +665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" style="32" min="1" max="1"/>
@@ -703,7 +700,7 @@
       </c>
       <c r="C4" s="32" t="inlineStr">
         <is>
-          <t>Hoang Phuc</t>
+          <t>[Enter your name]</t>
         </is>
       </c>
     </row>
@@ -715,7 +712,7 @@
       </c>
       <c r="C5" s="32" t="inlineStr">
         <is>
-          <t>QE...</t>
+          <t>Lê Đỗ Hoàng Phúc</t>
         </is>
       </c>
     </row>
@@ -727,7 +724,7 @@
       </c>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>CSD201</t>
+          <t>QE200057</t>
         </is>
       </c>
     </row>
@@ -739,7 +736,7 @@
       </c>
       <c r="C7" s="32" t="inlineStr">
         <is>
-          <t>Browser History</t>
+          <t>CSD201</t>
         </is>
       </c>
     </row>
@@ -773,7 +770,7 @@
           <t>Core Prompts Logged:</t>
         </is>
       </c>
-      <c r="C11" s="32" t="n">
+      <c r="C11" s="10" t="n">
         <v>6</v>
       </c>
     </row>
@@ -800,7 +797,7 @@
           <t>Hallucination Detected:</t>
         </is>
       </c>
-      <c r="C13" s="32" t="n">
+      <c r="C13" s="10" t="n">
         <v>3</v>
       </c>
     </row>
@@ -829,7 +826,7 @@
           <t>Purpose</t>
         </is>
       </c>
-      <c r="C16" s="38" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Frequency</t>
         </is>
@@ -928,6 +925,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="18.75" customHeight="1" s="35">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -946,7 +944,7 @@
           <t>Number of Prompts</t>
         </is>
       </c>
-      <c r="C23" s="38" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Required (Min)</t>
         </is>
@@ -1012,6 +1010,9 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
@@ -1127,7 +1128,7 @@
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>Tôi bác bỏ thiết kế này. Yêu cầu AI phân rã (Decomposition) bằng cách tách thành các hàm riêng biệt handleVisit(), handleBackward() gọi qua switch-case.</t>
+          <t>Bác bỏ thiết kế gộp chung. Yêu cầu AI phân rã (Decomposition) bằng cách tách thành các hàm xử lý riêng biệt như handleVisit(), handleBackward() gọi qua lệnh switch-case để đảm bảo tính module.</t>
         </is>
       </c>
       <c r="H4" s="24" t="inlineStr">
@@ -1169,7 +1170,7 @@
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>Tôi nhận ra dùng 2 Stacks tốn bộ nhớ. Tôi phản biện và chọn pattern Doubly Linked List kết hợp con trỏ current để đạt O(1) tuyệt đối.</t>
+          <t>Nhận thấy việc dùng 2 Stacks gây tốn bộ nhớ lưu trữ và tốn chi phí xử lý khi Pop/Push liên tục. Quyết định chọn cấu trúc Doubly Linked List kết hợp con trỏ current để đạt tốc độ di chuyển O(1) tuyệt đối.</t>
         </is>
       </c>
       <c r="H5" s="24" t="inlineStr">
@@ -1211,7 +1212,7 @@
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>Tôi nhận ra thời gian máy tính tự lấy được. Tôi viết hàm tự động gọi LocalDateTime.now() ẩn đi tham số này.</t>
+          <t>Nhận thấy thời gian là dữ liệu hệ thống tự lấy được. Tiến hành viết hàm tự động gọi LocalDateTime.now() nhằm ẩn đi tham số này, trừu tượng hóa và giảm bớt thao tác nhập liệu thừa thãi.</t>
         </is>
       </c>
       <c r="H6" s="24" t="inlineStr">
@@ -1253,7 +1254,7 @@
       </c>
       <c r="G7" s="24" t="inlineStr">
         <is>
-          <t>Tôi tự thiết kế thuật toán duyệt tuyến tính từ head. Chèn thêm điều kiện if (temp == current) để in ra &lt;&lt; CURRENT.</t>
+          <t>Thuật toán đếm của AI không xác định được vị trí trang hiện hành. Tự thiết kế thuật toán duyệt tuyến tính từ head, chèn thêm điều kiện if (temp == current) để in ra chuỗi &lt;&lt; CURRENT định vị trí.</t>
         </is>
       </c>
       <c r="H7" s="24" t="inlineStr">
@@ -1295,7 +1296,7 @@
       </c>
       <c r="G8" s="24" t="inlineStr">
         <is>
-          <t>Dùng try-catch cho lỗi Logic là sai. Tôi tự thiết kế thuật toán Guardrail ở dòng đầu: if (isEmpty()) return; giúp O(1) an toàn tuyệt đối.</t>
+          <t>Dùng try-catch để bắt lỗi logic NullPointerException là sai nguyên tắc. Tự thiết kế thuật toán Guardrail cực kỳ nhẹ ở dòng đầu: if (isEmpty()) return; giúp kiểm soát O(1) an toàn tuyệt đối.</t>
         </is>
       </c>
       <c r="H8" s="24" t="inlineStr">
@@ -1332,12 +1333,12 @@
       </c>
       <c r="F9" s="24" t="inlineStr">
         <is>
-          <t>AI 'tiện tay' sinh thêm hàm clearAllCache() và thuật toán getURLIndex(url) dùng vòng lặp O(N) để tìm kiếm.</t>
+          <t>AI sinh thêm hàm clearAllCache() và thuật toán getURLIndex(url) dùng vòng lặp O(N) để tìm kiếm.</t>
         </is>
       </c>
       <c r="G9" s="24" t="inlineStr">
         <is>
-          <t>Tôi bác bỏ hoàn toàn. Việc dùng vòng lặp tìm Index phá vỡ triết lý O(1). clearAllCache() cũng là thừa. Tôi dứt khoát xóa bỏ.</t>
+          <t>Bác bỏ hoàn toàn các hàm dư thừa. Việc dùng vòng lặp tìm Index phá vỡ triết lý O(1) của Linked List. Hàm clearAllCache() cũng không cần thiết. Dứt khoát xóa bỏ để tối ưu bộ nhớ.</t>
         </is>
       </c>
       <c r="H9" s="24" t="inlineStr">
@@ -1604,7 +1605,7 @@
       </c>
       <c r="F4" s="24" t="inlineStr">
         <is>
-          <t>Bác bỏ 2 Stacks. Tự triển khai bằng Doubly Linked List và con trỏ current.</t>
+          <t>Bác bỏ phương án 2 Stacks. Tự triển khai bằng Doubly Linked List và con trỏ current.</t>
         </is>
       </c>
     </row>
@@ -1636,7 +1637,7 @@
       </c>
       <c r="F5" s="28" t="inlineStr">
         <is>
-          <t>Bác bỏ tính năng này. Giữ nguyên việc thao tác bằng back() và forward.</t>
+          <t>Bác bỏ tính năng này. Giữ nguyên triết lý thao tác bằng back() và forward().</t>
         </is>
       </c>
     </row>
@@ -2224,6 +2225,8 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
+    <row r="24"/>
     <row r="25" ht="18.75" customHeight="1" s="35">
       <c r="A25" s="8" t="inlineStr">
         <is>
@@ -2268,17 +2271,17 @@
       </c>
       <c r="B28" s="24" t="inlineStr">
         <is>
-          <t>AI khuyên dùng 2 Stacks, nhưng 2 Stacks tốn gấp đôi bộ nhớ và thao tác Pop/Push liên tục không tối ưu. Em chốt dùng Doubly Linked List để đạt tốc độ O(1).</t>
+          <t>AI khuyên dùng 2 Stacks, nhưng 2 Stacks tốn bộ nhớ và thao tác Pop/Push liên tục không tối ưu. Do đó, chốt dùng Doubly Linked List để đạt tốc độ O(1).</t>
         </is>
       </c>
       <c r="C28" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> AI gen code tạo Stack&lt;Node&gt; past và Stack&lt;Node&gt; future.</t>
+          <t>Nhớ rõ: AI gen code tạo Stack&lt;Node&gt; past và Stack&lt;Node&gt; future.</t>
         </is>
       </c>
       <c r="D28" s="24" t="inlineStr">
         <is>
-          <t>Thể hiện ở class BrowserHistory chỉ dùng head, tail và current.</t>
+          <t>Thể hiện rõ ở class BrowserHistory chỉ dùng head, tail và current.</t>
         </is>
       </c>
     </row>
@@ -2290,17 +2293,17 @@
       </c>
       <c r="B29" s="24" t="inlineStr">
         <is>
-          <t>AI dùng vòng lặp đếm count bình thường. Em thiết kế lại vòng lặp kèm logic kiểm tra if (temp == current) để gắn mác &lt;&lt; CURRENT.</t>
+          <t>AI dùng vòng lặp đếm count bình thường không định vị được trang. Đã thiết kế lại vòng lặp kèm logic kiểm tra if (temp == current) để gắn mác &lt;&lt; CURRENT.</t>
         </is>
       </c>
       <c r="C29" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> AI chỉ gen được code in ra danh sách suông.</t>
+          <t>Nhớ rõ: AI chỉ gen được code in ra danh sách suông.</t>
         </is>
       </c>
       <c r="D29" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Nằm trực tiếp trong hàm showHistory() của em.</t>
+          <t>Nằm trực tiếp trong hàm showHistory() của module.</t>
         </is>
       </c>
     </row>
@@ -2312,17 +2315,17 @@
       </c>
       <c r="B30" s="24" t="inlineStr">
         <is>
-          <t>AI tự bịa hàm getURLIndex(url) chạy O(N). Em kiên quyết xóa bỏ vì thao tác trong Linked List tốn O(N) đi ngược lại triết lý tối ưu O(1).</t>
+          <t>AI tự sinh hàm getURLIndex(url) với thời gian chạy O(N). Kiên quyết xóa bỏ vì thao tác trong Linked List tốn O(N) đi ngược lại triết lý tối ưu O(1).</t>
         </is>
       </c>
       <c r="C30" s="24" t="inlineStr">
         <is>
-          <t>AI cung cấp hàm getURLIndex(String url) trong cấu trúc.</t>
+          <t>Nhớ rõ: AI cung cấp hàm getURLIndex(String url) trong cấu trúc.</t>
         </is>
       </c>
       <c r="D30" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Code của nhóm hoàn toàn sạch, không chứa hàm tìm kiếm O(N).</t>
+          <t>Code của nhóm hoàn toàn sạch, không chứa hàm tìm kiếm O(N).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync updated professional logs to main
</commit_message>
<xml_diff>
--- a/ai_logs/Phuc_AI_AuditLog.xlsx
+++ b/ai_logs/Phuc_AI_AuditLog.xlsx
@@ -211,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -298,9 +298,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -668,7 +665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" style="32" min="1" max="1"/>
@@ -703,7 +700,7 @@
       </c>
       <c r="C4" s="32" t="inlineStr">
         <is>
-          <t>Hoang Phuc</t>
+          <t>[Enter your name]</t>
         </is>
       </c>
     </row>
@@ -715,7 +712,7 @@
       </c>
       <c r="C5" s="32" t="inlineStr">
         <is>
-          <t>QE...</t>
+          <t>Lê Đỗ Hoàng Phúc</t>
         </is>
       </c>
     </row>
@@ -727,7 +724,7 @@
       </c>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>CSD201</t>
+          <t>QE200057</t>
         </is>
       </c>
     </row>
@@ -739,7 +736,7 @@
       </c>
       <c r="C7" s="32" t="inlineStr">
         <is>
-          <t>Browser History</t>
+          <t>CSD201</t>
         </is>
       </c>
     </row>
@@ -773,7 +770,7 @@
           <t>Core Prompts Logged:</t>
         </is>
       </c>
-      <c r="C11" s="32" t="n">
+      <c r="C11" s="10" t="n">
         <v>6</v>
       </c>
     </row>
@@ -800,7 +797,7 @@
           <t>Hallucination Detected:</t>
         </is>
       </c>
-      <c r="C13" s="32" t="n">
+      <c r="C13" s="10" t="n">
         <v>3</v>
       </c>
     </row>
@@ -829,7 +826,7 @@
           <t>Purpose</t>
         </is>
       </c>
-      <c r="C16" s="38" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Frequency</t>
         </is>
@@ -928,6 +925,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="18.75" customHeight="1" s="35">
       <c r="A22" s="8" t="inlineStr">
         <is>
@@ -946,7 +944,7 @@
           <t>Number of Prompts</t>
         </is>
       </c>
-      <c r="C23" s="38" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Required (Min)</t>
         </is>
@@ -1012,6 +1010,9 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
@@ -1127,7 +1128,7 @@
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>Tôi bác bỏ thiết kế này. Yêu cầu AI phân rã (Decomposition) bằng cách tách thành các hàm riêng biệt handleVisit(), handleBackward() gọi qua switch-case.</t>
+          <t>Bác bỏ thiết kế gộp chung. Yêu cầu AI phân rã (Decomposition) bằng cách tách thành các hàm xử lý riêng biệt như handleVisit(), handleBackward() gọi qua lệnh switch-case để đảm bảo tính module.</t>
         </is>
       </c>
       <c r="H4" s="24" t="inlineStr">
@@ -1169,7 +1170,7 @@
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>Tôi nhận ra dùng 2 Stacks tốn bộ nhớ. Tôi phản biện và chọn pattern Doubly Linked List kết hợp con trỏ current để đạt O(1) tuyệt đối.</t>
+          <t>Nhận thấy việc dùng 2 Stacks gây tốn bộ nhớ lưu trữ và tốn chi phí xử lý khi Pop/Push liên tục. Quyết định chọn cấu trúc Doubly Linked List kết hợp con trỏ current để đạt tốc độ di chuyển O(1) tuyệt đối.</t>
         </is>
       </c>
       <c r="H5" s="24" t="inlineStr">
@@ -1211,7 +1212,7 @@
       </c>
       <c r="G6" s="25" t="inlineStr">
         <is>
-          <t>Tôi nhận ra thời gian máy tính tự lấy được. Tôi viết hàm tự động gọi LocalDateTime.now() ẩn đi tham số này.</t>
+          <t>Nhận thấy thời gian là dữ liệu hệ thống tự lấy được. Tiến hành viết hàm tự động gọi LocalDateTime.now() nhằm ẩn đi tham số này, trừu tượng hóa và giảm bớt thao tác nhập liệu thừa thãi.</t>
         </is>
       </c>
       <c r="H6" s="24" t="inlineStr">
@@ -1253,7 +1254,7 @@
       </c>
       <c r="G7" s="24" t="inlineStr">
         <is>
-          <t>Tôi tự thiết kế thuật toán duyệt tuyến tính từ head. Chèn thêm điều kiện if (temp == current) để in ra &lt;&lt; CURRENT.</t>
+          <t>Thuật toán đếm của AI không xác định được vị trí trang hiện hành. Tự thiết kế thuật toán duyệt tuyến tính từ head, chèn thêm điều kiện if (temp == current) để in ra chuỗi &lt;&lt; CURRENT định vị trí.</t>
         </is>
       </c>
       <c r="H7" s="24" t="inlineStr">
@@ -1295,7 +1296,7 @@
       </c>
       <c r="G8" s="24" t="inlineStr">
         <is>
-          <t>Dùng try-catch cho lỗi Logic là sai. Tôi tự thiết kế thuật toán Guardrail ở dòng đầu: if (isEmpty()) return; giúp O(1) an toàn tuyệt đối.</t>
+          <t>Dùng try-catch để bắt lỗi logic NullPointerException là sai nguyên tắc. Tự thiết kế thuật toán Guardrail cực kỳ nhẹ ở dòng đầu: if (isEmpty()) return; giúp kiểm soát O(1) an toàn tuyệt đối.</t>
         </is>
       </c>
       <c r="H8" s="24" t="inlineStr">
@@ -1332,12 +1333,12 @@
       </c>
       <c r="F9" s="24" t="inlineStr">
         <is>
-          <t>AI 'tiện tay' sinh thêm hàm clearAllCache() và thuật toán getURLIndex(url) dùng vòng lặp O(N) để tìm kiếm.</t>
+          <t>AI sinh thêm hàm clearAllCache() và thuật toán getURLIndex(url) dùng vòng lặp O(N) để tìm kiếm.</t>
         </is>
       </c>
       <c r="G9" s="24" t="inlineStr">
         <is>
-          <t>Tôi bác bỏ hoàn toàn. Việc dùng vòng lặp tìm Index phá vỡ triết lý O(1). clearAllCache() cũng là thừa. Tôi dứt khoát xóa bỏ.</t>
+          <t>Bác bỏ hoàn toàn các hàm dư thừa. Việc dùng vòng lặp tìm Index phá vỡ triết lý O(1) của Linked List. Hàm clearAllCache() cũng không cần thiết. Dứt khoát xóa bỏ để tối ưu bộ nhớ.</t>
         </is>
       </c>
       <c r="H9" s="24" t="inlineStr">
@@ -1604,7 +1605,7 @@
       </c>
       <c r="F4" s="24" t="inlineStr">
         <is>
-          <t>Bác bỏ 2 Stacks. Tự triển khai bằng Doubly Linked List và con trỏ current.</t>
+          <t>Bác bỏ phương án 2 Stacks. Tự triển khai bằng Doubly Linked List và con trỏ current.</t>
         </is>
       </c>
     </row>
@@ -1636,7 +1637,7 @@
       </c>
       <c r="F5" s="28" t="inlineStr">
         <is>
-          <t>Bác bỏ tính năng này. Giữ nguyên việc thao tác bằng back() và forward.</t>
+          <t>Bác bỏ tính năng này. Giữ nguyên triết lý thao tác bằng back() và forward().</t>
         </is>
       </c>
     </row>
@@ -2224,6 +2225,8 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
+    <row r="24"/>
     <row r="25" ht="18.75" customHeight="1" s="35">
       <c r="A25" s="8" t="inlineStr">
         <is>
@@ -2268,17 +2271,17 @@
       </c>
       <c r="B28" s="24" t="inlineStr">
         <is>
-          <t>AI khuyên dùng 2 Stacks, nhưng 2 Stacks tốn gấp đôi bộ nhớ và thao tác Pop/Push liên tục không tối ưu. Em chốt dùng Doubly Linked List để đạt tốc độ O(1).</t>
+          <t>AI khuyên dùng 2 Stacks, nhưng 2 Stacks tốn bộ nhớ và thao tác Pop/Push liên tục không tối ưu. Do đó, chốt dùng Doubly Linked List để đạt tốc độ O(1).</t>
         </is>
       </c>
       <c r="C28" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> AI gen code tạo Stack&lt;Node&gt; past và Stack&lt;Node&gt; future.</t>
+          <t>Nhớ rõ: AI gen code tạo Stack&lt;Node&gt; past và Stack&lt;Node&gt; future.</t>
         </is>
       </c>
       <c r="D28" s="24" t="inlineStr">
         <is>
-          <t>Thể hiện ở class BrowserHistory chỉ dùng head, tail và current.</t>
+          <t>Thể hiện rõ ở class BrowserHistory chỉ dùng head, tail và current.</t>
         </is>
       </c>
     </row>
@@ -2290,17 +2293,17 @@
       </c>
       <c r="B29" s="24" t="inlineStr">
         <is>
-          <t>AI dùng vòng lặp đếm count bình thường. Em thiết kế lại vòng lặp kèm logic kiểm tra if (temp == current) để gắn mác &lt;&lt; CURRENT.</t>
+          <t>AI dùng vòng lặp đếm count bình thường không định vị được trang. Đã thiết kế lại vòng lặp kèm logic kiểm tra if (temp == current) để gắn mác &lt;&lt; CURRENT.</t>
         </is>
       </c>
       <c r="C29" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> AI chỉ gen được code in ra danh sách suông.</t>
+          <t>Nhớ rõ: AI chỉ gen được code in ra danh sách suông.</t>
         </is>
       </c>
       <c r="D29" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Nằm trực tiếp trong hàm showHistory() của em.</t>
+          <t>Nằm trực tiếp trong hàm showHistory() của module.</t>
         </is>
       </c>
     </row>
@@ -2312,17 +2315,17 @@
       </c>
       <c r="B30" s="24" t="inlineStr">
         <is>
-          <t>AI tự bịa hàm getURLIndex(url) chạy O(N). Em kiên quyết xóa bỏ vì thao tác trong Linked List tốn O(N) đi ngược lại triết lý tối ưu O(1).</t>
+          <t>AI tự sinh hàm getURLIndex(url) với thời gian chạy O(N). Kiên quyết xóa bỏ vì thao tác trong Linked List tốn O(N) đi ngược lại triết lý tối ưu O(1).</t>
         </is>
       </c>
       <c r="C30" s="24" t="inlineStr">
         <is>
-          <t>AI cung cấp hàm getURLIndex(String url) trong cấu trúc.</t>
+          <t>Nhớ rõ: AI cung cấp hàm getURLIndex(String url) trong cấu trúc.</t>
         </is>
       </c>
       <c r="D30" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Code của nhóm hoàn toàn sạch, không chứa hàm tìm kiếm O(N).</t>
+          <t>Code của nhóm hoàn toàn sạch, không chứa hàm tìm kiếm O(N).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace 'Bac bo' with 'Bo' for softer tone
</commit_message>
<xml_diff>
--- a/ai_logs/Phuc_AI_AuditLog.xlsx
+++ b/ai_logs/Phuc_AI_AuditLog.xlsx
@@ -665,7 +665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" style="32" min="1" max="1"/>
@@ -1010,9 +1010,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
@@ -1128,7 +1125,7 @@
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>Bác bỏ thiết kế gộp chung. Yêu cầu AI phân rã (Decomposition) bằng cách tách thành các hàm xử lý riêng biệt như handleVisit(), handleBackward() gọi qua lệnh switch-case để đảm bảo tính module.</t>
+          <t>Bỏ thiết kế gộp chung. Yêu cầu AI phân rã (Decomposition) bằng cách tách thành các hàm xử lý riêng biệt như handleVisit(), handleBackward() gọi qua lệnh switch-case để đảm bảo tính module.</t>
         </is>
       </c>
       <c r="H4" s="24" t="inlineStr">
@@ -1338,7 +1335,7 @@
       </c>
       <c r="G9" s="24" t="inlineStr">
         <is>
-          <t>Bác bỏ hoàn toàn các hàm dư thừa. Việc dùng vòng lặp tìm Index phá vỡ triết lý O(1) của Linked List. Hàm clearAllCache() cũng không cần thiết. Dứt khoát xóa bỏ để tối ưu bộ nhớ.</t>
+          <t>Bỏ hoàn toàn các hàm dư thừa. Việc dùng vòng lặp tìm Index phá vỡ triết lý O(1) của Linked List. Hàm clearAllCache() cũng không cần thiết. Dứt khoát xóa bỏ để tối ưu bộ nhớ.</t>
         </is>
       </c>
       <c r="H9" s="24" t="inlineStr">
@@ -1605,7 +1602,7 @@
       </c>
       <c r="F4" s="24" t="inlineStr">
         <is>
-          <t>Bác bỏ phương án 2 Stacks. Tự triển khai bằng Doubly Linked List và con trỏ current.</t>
+          <t>Bỏ phương án 2 Stacks. Tự triển khai bằng Doubly Linked List và con trỏ current.</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1634,7 @@
       </c>
       <c r="F5" s="28" t="inlineStr">
         <is>
-          <t>Bác bỏ tính năng này. Giữ nguyên triết lý thao tác bằng back() và forward().</t>
+          <t>Bỏ tính năng này. Giữ nguyên triết lý thao tác bằng back() và forward().</t>
         </is>
       </c>
     </row>
@@ -1817,6 +1814,11 @@
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n"/>
     </row>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
     <row r="30" ht="18.75" customHeight="1" s="35">
       <c r="A30" s="1" t="inlineStr">
         <is>
@@ -1966,6 +1968,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="18.75" customHeight="1" s="35">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -2085,6 +2088,7 @@
       </c>
       <c r="D10" s="17" t="n"/>
     </row>
+    <row r="11"/>
     <row r="12" ht="18.75" customHeight="1" s="35">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -2204,6 +2208,7 @@
       </c>
       <c r="D18" s="17" t="n"/>
     </row>
+    <row r="19"/>
     <row r="20" ht="15.75" customHeight="1" s="35">
       <c r="A20" s="18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sync softer tone to main
</commit_message>
<xml_diff>
--- a/ai_logs/Phuc_AI_AuditLog.xlsx
+++ b/ai_logs/Phuc_AI_AuditLog.xlsx
@@ -665,7 +665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" style="32" min="1" max="1"/>
@@ -1010,9 +1010,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
@@ -1128,7 +1125,7 @@
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>Bác bỏ thiết kế gộp chung. Yêu cầu AI phân rã (Decomposition) bằng cách tách thành các hàm xử lý riêng biệt như handleVisit(), handleBackward() gọi qua lệnh switch-case để đảm bảo tính module.</t>
+          <t>Bỏ thiết kế gộp chung. Yêu cầu AI phân rã (Decomposition) bằng cách tách thành các hàm xử lý riêng biệt như handleVisit(), handleBackward() gọi qua lệnh switch-case để đảm bảo tính module.</t>
         </is>
       </c>
       <c r="H4" s="24" t="inlineStr">
@@ -1338,7 +1335,7 @@
       </c>
       <c r="G9" s="24" t="inlineStr">
         <is>
-          <t>Bác bỏ hoàn toàn các hàm dư thừa. Việc dùng vòng lặp tìm Index phá vỡ triết lý O(1) của Linked List. Hàm clearAllCache() cũng không cần thiết. Dứt khoát xóa bỏ để tối ưu bộ nhớ.</t>
+          <t>Bỏ hoàn toàn các hàm dư thừa. Việc dùng vòng lặp tìm Index phá vỡ triết lý O(1) của Linked List. Hàm clearAllCache() cũng không cần thiết. Dứt khoát xóa bỏ để tối ưu bộ nhớ.</t>
         </is>
       </c>
       <c r="H9" s="24" t="inlineStr">
@@ -1605,7 +1602,7 @@
       </c>
       <c r="F4" s="24" t="inlineStr">
         <is>
-          <t>Bác bỏ phương án 2 Stacks. Tự triển khai bằng Doubly Linked List và con trỏ current.</t>
+          <t>Bỏ phương án 2 Stacks. Tự triển khai bằng Doubly Linked List và con trỏ current.</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1634,7 @@
       </c>
       <c r="F5" s="28" t="inlineStr">
         <is>
-          <t>Bác bỏ tính năng này. Giữ nguyên triết lý thao tác bằng back() và forward().</t>
+          <t>Bỏ tính năng này. Giữ nguyên triết lý thao tác bằng back() và forward().</t>
         </is>
       </c>
     </row>
@@ -1817,6 +1814,11 @@
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n"/>
     </row>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
     <row r="30" ht="18.75" customHeight="1" s="35">
       <c r="A30" s="1" t="inlineStr">
         <is>
@@ -1966,6 +1968,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="18.75" customHeight="1" s="35">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -2085,6 +2088,7 @@
       </c>
       <c r="D10" s="17" t="n"/>
     </row>
+    <row r="11"/>
     <row r="12" ht="18.75" customHeight="1" s="35">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -2204,6 +2208,7 @@
       </c>
       <c r="D18" s="17" t="n"/>
     </row>
+    <row r="19"/>
     <row r="20" ht="15.75" customHeight="1" s="35">
       <c r="A20" s="18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update DTC Component table numbers and remove yellow fill
</commit_message>
<xml_diff>
--- a/ai_logs/Phuc_AI_AuditLog.xlsx
+++ b/ai_logs/Phuc_AI_AuditLog.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1815" yWindow="1815" windowWidth="28800" windowHeight="15225" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="360" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Metadata &amp; Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -288,9 +288,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -298,6 +295,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -665,7 +665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" style="32" min="1" max="1"/>
@@ -673,8 +673,8 @@
     <col width="15" customWidth="1" style="32" min="3" max="3"/>
     <col width="30" customWidth="1" style="32" min="4" max="4"/>
     <col width="20" customWidth="1" style="32" min="5" max="6"/>
-    <col width="8.7109375" customWidth="1" style="32" min="7" max="9"/>
-    <col width="8.7109375" customWidth="1" style="32" min="10" max="16384"/>
+    <col width="8.7109375" customWidth="1" style="32" min="7" max="10"/>
+    <col width="8.7109375" customWidth="1" style="32" min="11" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -684,8 +684,7 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
-    <row r="3" ht="18.75" customHeight="1" s="35">
+    <row r="3" ht="18.75" customHeight="1" s="34">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>STUDENT INFORMATION</t>
@@ -700,7 +699,7 @@
       </c>
       <c r="C4" s="32" t="inlineStr">
         <is>
-          <t>[Enter your name]</t>
+          <t>Lê Đỗ Hoàng Phúc</t>
         </is>
       </c>
     </row>
@@ -712,7 +711,7 @@
       </c>
       <c r="C5" s="32" t="inlineStr">
         <is>
-          <t>Lê Đỗ Hoàng Phúc</t>
+          <t>QE200057</t>
         </is>
       </c>
     </row>
@@ -724,7 +723,7 @@
       </c>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>QE200057</t>
+          <t>CSD201</t>
         </is>
       </c>
     </row>
@@ -734,20 +733,14 @@
           <t>Assignment:</t>
         </is>
       </c>
-      <c r="C7" s="32" t="inlineStr">
-        <is>
-          <t>CSD201</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Browser History</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18.75" customHeight="1" s="35">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Browser History and Cache Navigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9" ht="18.75" customHeight="1" s="34">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>AI USAGE SUMMARY</t>
@@ -808,7 +801,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="18.75" customHeight="1" s="35">
+    <row r="15" ht="18.75" customHeight="1" s="34">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>AI TOOLS USED</t>
@@ -859,7 +852,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1" s="35">
+    <row r="18" ht="30" customHeight="1" s="34">
       <c r="A18" s="7" t="inlineStr">
         <is>
           <t>Claude</t>
@@ -881,7 +874,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1" s="35">
+    <row r="19" ht="30" customHeight="1" s="34">
       <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Gemini</t>
@@ -903,7 +896,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1" s="35">
+    <row r="20" ht="30" customHeight="1" s="34">
       <c r="A20" s="7" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -926,14 +919,14 @@
       </c>
     </row>
     <row r="21"/>
-    <row r="22" ht="18.75" customHeight="1" s="35">
+    <row r="22" ht="18.75" customHeight="1" s="34">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>CORE PROMPTS DISTRIBUTION BY DTC COMPONENT</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="28.5" customHeight="1" s="35">
+    <row r="23" ht="28.5" customHeight="1" s="34">
       <c r="A23" s="6" t="inlineStr">
         <is>
           <t>DTC Component</t>
@@ -956,8 +949,8 @@
           <t>Decomposition</t>
         </is>
       </c>
-      <c r="B24" s="13" t="n">
-        <v>0</v>
+      <c r="B24" s="14" t="n">
+        <v>1</v>
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
@@ -971,8 +964,8 @@
           <t>Pattern Recognition</t>
         </is>
       </c>
-      <c r="B25" s="13" t="n">
-        <v>0</v>
+      <c r="B25" s="14" t="n">
+        <v>1</v>
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
@@ -986,8 +979,8 @@
           <t>Abstraction</t>
         </is>
       </c>
-      <c r="B26" s="13" t="n">
-        <v>0</v>
+      <c r="B26" s="14" t="n">
+        <v>1</v>
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
@@ -1001,8 +994,8 @@
           <t>Algorithms</t>
         </is>
       </c>
-      <c r="B27" s="13" t="n">
-        <v>0</v>
+      <c r="B27" s="14" t="n">
+        <v>3</v>
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
@@ -1010,6 +1003,19 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
@@ -1027,13 +1033,13 @@
   <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" style="35" min="1" max="1"/>
-    <col width="18" customWidth="1" style="35" min="2" max="3"/>
-    <col width="25" customWidth="1" style="35" min="4" max="4"/>
-    <col width="30" customWidth="1" style="35" min="5" max="5"/>
-    <col width="35" customWidth="1" style="35" min="6" max="6"/>
-    <col width="50" customWidth="1" style="35" min="7" max="7"/>
-    <col width="26.85546875" customWidth="1" style="35" min="8" max="8"/>
+    <col width="8" customWidth="1" style="34" min="1" max="1"/>
+    <col width="18" customWidth="1" style="34" min="2" max="3"/>
+    <col width="25" customWidth="1" style="34" min="4" max="4"/>
+    <col width="30" customWidth="1" style="34" min="5" max="5"/>
+    <col width="35" customWidth="1" style="34" min="6" max="6"/>
+    <col width="50" customWidth="1" style="34" min="7" max="7"/>
+    <col width="26.85546875" customWidth="1" style="34" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1043,14 +1049,14 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1" s="35">
-      <c r="A2" s="34" t="inlineStr">
+    <row r="2" ht="30" customHeight="1" s="34">
+      <c r="A2" s="33" t="inlineStr">
         <is>
           <t>INSTRUCTIONS: Chỉ ghi CORE PROMPTS (Decision/Problem-Solving/Verification). Mỗi entry phải trả lời đầy đủ 4 câu hỏi trong Human Delta.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="39.95" customHeight="1" s="35">
+    <row r="3" ht="39.95" customHeight="1" s="34">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Entry #</t>
@@ -1092,7 +1098,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="99.95" customHeight="1" s="35">
+    <row r="4" ht="99.95" customHeight="1" s="34">
       <c r="A4" s="23" t="inlineStr">
         <is>
           <t>001</t>
@@ -1134,7 +1140,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="99.95" customHeight="1" s="35" thickBot="1">
+    <row r="5" ht="99.95" customHeight="1" s="34" thickBot="1">
       <c r="A5" s="23" t="inlineStr">
         <is>
           <t>002</t>
@@ -1176,7 +1182,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="80.09999999999999" customHeight="1" s="35" thickBot="1">
+    <row r="6" ht="80.09999999999999" customHeight="1" s="34" thickBot="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
           <t>003</t>
@@ -1315,7 +1321,7 @@
       </c>
       <c r="C9" s="24" t="inlineStr">
         <is>
-          <t>Refactoring</t>
+          <t>Algorithms</t>
         </is>
       </c>
       <c r="D9" s="24" t="inlineStr">
@@ -1344,7 +1350,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="10" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A10" s="3" t="n"/>
       <c r="B10" s="3" t="n"/>
       <c r="C10" s="3" t="n"/>
@@ -1354,7 +1360,7 @@
       <c r="G10" s="3" t="n"/>
       <c r="H10" s="3" t="n"/>
     </row>
-    <row r="11" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="11" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A11" s="3" t="n"/>
       <c r="B11" s="3" t="n"/>
       <c r="C11" s="3" t="n"/>
@@ -1364,7 +1370,7 @@
       <c r="G11" s="3" t="n"/>
       <c r="H11" s="3" t="n"/>
     </row>
-    <row r="12" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="12" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A12" s="3" t="n"/>
       <c r="B12" s="3" t="n"/>
       <c r="C12" s="3" t="n"/>
@@ -1374,7 +1380,7 @@
       <c r="G12" s="3" t="n"/>
       <c r="H12" s="3" t="n"/>
     </row>
-    <row r="13" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="13" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A13" s="3" t="n"/>
       <c r="B13" s="3" t="n"/>
       <c r="C13" s="3" t="n"/>
@@ -1384,7 +1390,7 @@
       <c r="G13" s="3" t="n"/>
       <c r="H13" s="3" t="n"/>
     </row>
-    <row r="14" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="14" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A14" s="3" t="n"/>
       <c r="B14" s="3" t="n"/>
       <c r="C14" s="3" t="n"/>
@@ -1394,7 +1400,7 @@
       <c r="G14" s="3" t="n"/>
       <c r="H14" s="3" t="n"/>
     </row>
-    <row r="15" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="15" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A15" s="3" t="n"/>
       <c r="B15" s="3" t="n"/>
       <c r="C15" s="3" t="n"/>
@@ -1404,7 +1410,7 @@
       <c r="G15" s="3" t="n"/>
       <c r="H15" s="3" t="n"/>
     </row>
-    <row r="16" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="16" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A16" s="3" t="n"/>
       <c r="B16" s="3" t="n"/>
       <c r="C16" s="3" t="n"/>
@@ -1414,7 +1420,7 @@
       <c r="G16" s="3" t="n"/>
       <c r="H16" s="3" t="n"/>
     </row>
-    <row r="17" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="17" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A17" s="3" t="n"/>
       <c r="B17" s="3" t="n"/>
       <c r="C17" s="3" t="n"/>
@@ -1424,7 +1430,7 @@
       <c r="G17" s="3" t="n"/>
       <c r="H17" s="3" t="n"/>
     </row>
-    <row r="18" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="18" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A18" s="3" t="n"/>
       <c r="B18" s="3" t="n"/>
       <c r="C18" s="3" t="n"/>
@@ -1434,7 +1440,7 @@
       <c r="G18" s="3" t="n"/>
       <c r="H18" s="3" t="n"/>
     </row>
-    <row r="19" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="19" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A19" s="3" t="n"/>
       <c r="B19" s="3" t="n"/>
       <c r="C19" s="3" t="n"/>
@@ -1444,7 +1450,7 @@
       <c r="G19" s="3" t="n"/>
       <c r="H19" s="3" t="n"/>
     </row>
-    <row r="20" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="20" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A20" s="3" t="n"/>
       <c r="B20" s="3" t="n"/>
       <c r="C20" s="3" t="n"/>
@@ -1454,7 +1460,7 @@
       <c r="G20" s="3" t="n"/>
       <c r="H20" s="3" t="n"/>
     </row>
-    <row r="21" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="21" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A21" s="3" t="n"/>
       <c r="B21" s="3" t="n"/>
       <c r="C21" s="3" t="n"/>
@@ -1464,7 +1470,7 @@
       <c r="G21" s="3" t="n"/>
       <c r="H21" s="3" t="n"/>
     </row>
-    <row r="22" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="22" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A22" s="3" t="n"/>
       <c r="B22" s="3" t="n"/>
       <c r="C22" s="3" t="n"/>
@@ -1474,7 +1480,7 @@
       <c r="G22" s="3" t="n"/>
       <c r="H22" s="3" t="n"/>
     </row>
-    <row r="23" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="23" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A23" s="3" t="n"/>
       <c r="B23" s="3" t="n"/>
       <c r="C23" s="3" t="n"/>
@@ -1484,7 +1490,7 @@
       <c r="G23" s="3" t="n"/>
       <c r="H23" s="3" t="n"/>
     </row>
-    <row r="24" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="24" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A24" s="3" t="n"/>
       <c r="B24" s="3" t="n"/>
       <c r="C24" s="3" t="n"/>
@@ -1494,7 +1500,7 @@
       <c r="G24" s="3" t="n"/>
       <c r="H24" s="3" t="n"/>
     </row>
-    <row r="25" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="25" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A25" s="3" t="n"/>
       <c r="B25" s="3" t="n"/>
       <c r="C25" s="3" t="n"/>
@@ -1523,26 +1529,26 @@
   <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" style="35" min="1" max="1"/>
-    <col width="22" customWidth="1" style="35" min="2" max="2"/>
-    <col width="30" customWidth="1" style="35" min="3" max="6"/>
+    <col width="12" customWidth="1" style="34" min="1" max="1"/>
+    <col width="22" customWidth="1" style="34" min="2" max="2"/>
+    <col width="30" customWidth="1" style="34" min="3" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="37" t="inlineStr">
+      <c r="A1" s="36" t="inlineStr">
         <is>
           <t>HALLUCINATION DETECTION LOG (BẮT BUỘC)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="36" t="inlineStr">
+      <c r="A2" s="35" t="inlineStr">
         <is>
           <t>MỖI PROJECT PHẢI PHÁT HIỆN ÍT NHẤT: Lab (≥1), Assignment (≥2), Project (≥3) cases hallucination</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="39.95" customHeight="1" s="35">
+    <row r="3" ht="39.95" customHeight="1" s="34">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Entry # (from Sheet 2)</t>
@@ -1574,7 +1580,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1" s="35">
+    <row r="4" ht="60" customHeight="1" s="34">
       <c r="A4" s="26" t="inlineStr">
         <is>
           <t>001</t>
@@ -1606,7 +1612,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1" s="35">
+    <row r="5" ht="30" customHeight="1" s="34">
       <c r="A5" s="27" t="inlineStr">
         <is>
           <t>002</t>
@@ -1638,7 +1644,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1" s="35">
+    <row r="6" ht="60" customHeight="1" s="34">
       <c r="A6" s="27" t="inlineStr">
         <is>
           <t>003</t>
@@ -1670,7 +1676,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1" s="35">
+    <row r="7" ht="60" customHeight="1" s="34">
       <c r="A7" s="3" t="n"/>
       <c r="B7" s="3" t="n"/>
       <c r="C7" s="3" t="n"/>
@@ -1678,7 +1684,7 @@
       <c r="E7" s="3" t="n"/>
       <c r="F7" s="3" t="n"/>
     </row>
-    <row r="8" ht="60" customHeight="1" s="35">
+    <row r="8" ht="60" customHeight="1" s="34">
       <c r="A8" s="3" t="n"/>
       <c r="B8" s="3" t="n"/>
       <c r="C8" s="3" t="n"/>
@@ -1686,7 +1692,7 @@
       <c r="E8" s="3" t="n"/>
       <c r="F8" s="3" t="n"/>
     </row>
-    <row r="9" ht="60" customHeight="1" s="35">
+    <row r="9" ht="60" customHeight="1" s="34">
       <c r="A9" s="3" t="n"/>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="3" t="n"/>
@@ -1694,7 +1700,7 @@
       <c r="E9" s="3" t="n"/>
       <c r="F9" s="3" t="n"/>
     </row>
-    <row r="10" ht="60" customHeight="1" s="35">
+    <row r="10" ht="60" customHeight="1" s="34">
       <c r="A10" s="3" t="n"/>
       <c r="B10" s="3" t="n"/>
       <c r="C10" s="3" t="n"/>
@@ -1702,7 +1708,7 @@
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="3" t="n"/>
     </row>
-    <row r="11" ht="60" customHeight="1" s="35">
+    <row r="11" ht="60" customHeight="1" s="34">
       <c r="A11" s="3" t="n"/>
       <c r="B11" s="3" t="n"/>
       <c r="C11" s="3" t="n"/>
@@ -1710,7 +1716,7 @@
       <c r="E11" s="3" t="n"/>
       <c r="F11" s="3" t="n"/>
     </row>
-    <row r="12" ht="60" customHeight="1" s="35">
+    <row r="12" ht="60" customHeight="1" s="34">
       <c r="A12" s="3" t="n"/>
       <c r="B12" s="3" t="n"/>
       <c r="C12" s="3" t="n"/>
@@ -1718,7 +1724,7 @@
       <c r="E12" s="3" t="n"/>
       <c r="F12" s="3" t="n"/>
     </row>
-    <row r="13" ht="60" customHeight="1" s="35">
+    <row r="13" ht="60" customHeight="1" s="34">
       <c r="A13" s="3" t="n"/>
       <c r="B13" s="3" t="n"/>
       <c r="C13" s="3" t="n"/>
@@ -1726,7 +1732,7 @@
       <c r="E13" s="3" t="n"/>
       <c r="F13" s="3" t="n"/>
     </row>
-    <row r="14" ht="60" customHeight="1" s="35">
+    <row r="14" ht="60" customHeight="1" s="34">
       <c r="A14" s="3" t="n"/>
       <c r="B14" s="3" t="n"/>
       <c r="C14" s="3" t="n"/>
@@ -1734,7 +1740,7 @@
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="3" t="n"/>
     </row>
-    <row r="15" ht="60" customHeight="1" s="35">
+    <row r="15" ht="60" customHeight="1" s="34">
       <c r="A15" s="3" t="n"/>
       <c r="B15" s="3" t="n"/>
       <c r="C15" s="3" t="n"/>
@@ -1742,7 +1748,7 @@
       <c r="E15" s="3" t="n"/>
       <c r="F15" s="3" t="n"/>
     </row>
-    <row r="16" ht="60" customHeight="1" s="35">
+    <row r="16" ht="60" customHeight="1" s="34">
       <c r="A16" s="3" t="n"/>
       <c r="B16" s="3" t="n"/>
       <c r="C16" s="3" t="n"/>
@@ -1750,7 +1756,7 @@
       <c r="E16" s="3" t="n"/>
       <c r="F16" s="3" t="n"/>
     </row>
-    <row r="17" ht="60" customHeight="1" s="35">
+    <row r="17" ht="60" customHeight="1" s="34">
       <c r="A17" s="3" t="n"/>
       <c r="B17" s="3" t="n"/>
       <c r="C17" s="3" t="n"/>
@@ -1758,7 +1764,7 @@
       <c r="E17" s="3" t="n"/>
       <c r="F17" s="3" t="n"/>
     </row>
-    <row r="18" ht="60" customHeight="1" s="35">
+    <row r="18" ht="60" customHeight="1" s="34">
       <c r="A18" s="3" t="n"/>
       <c r="B18" s="3" t="n"/>
       <c r="C18" s="3" t="n"/>
@@ -1766,7 +1772,7 @@
       <c r="E18" s="3" t="n"/>
       <c r="F18" s="3" t="n"/>
     </row>
-    <row r="19" ht="60" customHeight="1" s="35">
+    <row r="19" ht="60" customHeight="1" s="34">
       <c r="A19" s="3" t="n"/>
       <c r="B19" s="3" t="n"/>
       <c r="C19" s="3" t="n"/>
@@ -1774,7 +1780,7 @@
       <c r="E19" s="3" t="n"/>
       <c r="F19" s="3" t="n"/>
     </row>
-    <row r="20" ht="60" customHeight="1" s="35">
+    <row r="20" ht="60" customHeight="1" s="34">
       <c r="A20" s="3" t="n"/>
       <c r="B20" s="3" t="n"/>
       <c r="C20" s="3" t="n"/>
@@ -1782,7 +1788,7 @@
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n"/>
     </row>
-    <row r="21" ht="60" customHeight="1" s="35">
+    <row r="21" ht="60" customHeight="1" s="34">
       <c r="A21" s="3" t="n"/>
       <c r="B21" s="3" t="n"/>
       <c r="C21" s="3" t="n"/>
@@ -1790,7 +1796,7 @@
       <c r="E21" s="3" t="n"/>
       <c r="F21" s="3" t="n"/>
     </row>
-    <row r="22" ht="60" customHeight="1" s="35">
+    <row r="22" ht="60" customHeight="1" s="34">
       <c r="A22" s="3" t="n"/>
       <c r="B22" s="3" t="n"/>
       <c r="C22" s="3" t="n"/>
@@ -1798,7 +1804,7 @@
       <c r="E22" s="3" t="n"/>
       <c r="F22" s="3" t="n"/>
     </row>
-    <row r="23" ht="60" customHeight="1" s="35">
+    <row r="23" ht="60" customHeight="1" s="34">
       <c r="A23" s="3" t="n"/>
       <c r="B23" s="3" t="n"/>
       <c r="C23" s="3" t="n"/>
@@ -1806,7 +1812,7 @@
       <c r="E23" s="3" t="n"/>
       <c r="F23" s="3" t="n"/>
     </row>
-    <row r="24" ht="60" customHeight="1" s="35">
+    <row r="24" ht="60" customHeight="1" s="34">
       <c r="A24" s="3" t="n"/>
       <c r="B24" s="3" t="n"/>
       <c r="C24" s="3" t="n"/>
@@ -1814,12 +1820,7 @@
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n"/>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30" ht="18.75" customHeight="1" s="35">
+    <row r="30" ht="18.75" customHeight="1" s="34">
       <c r="A30" s="1" t="inlineStr">
         <is>
           <t>HALLUCINATION TYPES REFERENCE:</t>
@@ -1843,7 +1844,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1" s="35">
+    <row r="32" ht="30" customHeight="1" s="34">
       <c r="A32" s="3" t="inlineStr">
         <is>
           <t>Fabrication</t>
@@ -1860,7 +1861,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="30" customHeight="1" s="35">
+    <row r="33" ht="30" customHeight="1" s="34">
       <c r="A33" s="3" t="inlineStr">
         <is>
           <t>Oversimplification</t>
@@ -1877,7 +1878,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="30" customHeight="1" s="35">
+    <row r="34" ht="30" customHeight="1" s="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
           <t>Logic Error</t>
@@ -1894,7 +1895,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="30" customHeight="1" s="35">
+    <row r="35" ht="30" customHeight="1" s="34">
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t>Outdated Info</t>
@@ -1911,7 +1912,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="45" customHeight="1" s="35">
+    <row r="36" ht="45" customHeight="1" s="34">
       <c r="A36" s="3" t="inlineStr">
         <is>
           <t>Context Misunderstanding</t>
@@ -1950,8 +1951,8 @@
     <col width="60" customWidth="1" style="32" min="2" max="2"/>
     <col width="10" customWidth="1" style="32" min="3" max="3"/>
     <col width="30" customWidth="1" style="32" min="4" max="4"/>
-    <col width="8.7109375" customWidth="1" style="32" min="5" max="7"/>
-    <col width="8.7109375" customWidth="1" style="32" min="8" max="16384"/>
+    <col width="8.7109375" customWidth="1" style="32" min="5" max="8"/>
+    <col width="8.7109375" customWidth="1" style="32" min="9" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1962,14 +1963,13 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="33" t="inlineStr">
+      <c r="A2" s="37" t="inlineStr">
         <is>
           <t>Kiểm tra kỹ trước khi nộp. MỖI ENTRY phải pass ≥4/5 tiêu chí dưới đây.</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4" ht="18.75" customHeight="1" s="35">
+    <row r="4" ht="18.75" customHeight="1" s="34">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>A. KIỂM TRA CHẤT LƯỢNG MỖI ENTRY (Pass ≥4/5)</t>
@@ -2088,8 +2088,7 @@
       </c>
       <c r="D10" s="17" t="n"/>
     </row>
-    <row r="11"/>
-    <row r="12" ht="18.75" customHeight="1" s="35">
+    <row r="12" ht="18.75" customHeight="1" s="34">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>B. KIỂM TRA TỔNG THỂ LOG</t>
@@ -2208,8 +2207,7 @@
       </c>
       <c r="D18" s="17" t="n"/>
     </row>
-    <row r="19"/>
-    <row r="20" ht="15.75" customHeight="1" s="35">
+    <row r="20" ht="15.75" customHeight="1" s="34">
       <c r="A20" s="18" t="inlineStr">
         <is>
           <t>⚠️ LƯU Ý QUAN TRỌNG:</t>
@@ -2230,9 +2228,7 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25" ht="18.75" customHeight="1" s="35">
+    <row r="25" ht="18.75" customHeight="1" s="34">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>C. CHUẨN BỊ CHO ORAL VIVAS (Q&amp;A)</t>
@@ -2246,7 +2242,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="57" customHeight="1" s="35">
+    <row r="27" ht="57" customHeight="1" s="34">
       <c r="A27" s="21" t="inlineStr">
         <is>
           <t>Entry #</t>
@@ -2268,7 +2264,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="120" customHeight="1" s="35">
+    <row r="28" ht="120" customHeight="1" s="34">
       <c r="A28" s="23" t="inlineStr">
         <is>
           <t>002</t>
@@ -2290,7 +2286,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="75" customHeight="1" s="35">
+    <row r="29" ht="75" customHeight="1" s="34">
       <c r="A29" s="23" t="inlineStr">
         <is>
           <t>004</t>
@@ -2312,7 +2308,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="90" customHeight="1" s="35">
+    <row r="30" ht="90" customHeight="1" s="34">
       <c r="A30" s="23" t="inlineStr">
         <is>
           <t>006</t>

</xml_diff>

<commit_message>
Sync updated DTC Component table to main
</commit_message>
<xml_diff>
--- a/ai_logs/Phuc_AI_AuditLog.xlsx
+++ b/ai_logs/Phuc_AI_AuditLog.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1815" yWindow="1815" windowWidth="28800" windowHeight="15225" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="360" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Metadata &amp; Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -288,9 +288,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -298,6 +295,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -665,7 +665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" style="32" min="1" max="1"/>
@@ -673,8 +673,8 @@
     <col width="15" customWidth="1" style="32" min="3" max="3"/>
     <col width="30" customWidth="1" style="32" min="4" max="4"/>
     <col width="20" customWidth="1" style="32" min="5" max="6"/>
-    <col width="8.7109375" customWidth="1" style="32" min="7" max="9"/>
-    <col width="8.7109375" customWidth="1" style="32" min="10" max="16384"/>
+    <col width="8.7109375" customWidth="1" style="32" min="7" max="10"/>
+    <col width="8.7109375" customWidth="1" style="32" min="11" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -684,8 +684,7 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
-    <row r="3" ht="18.75" customHeight="1" s="35">
+    <row r="3" ht="18.75" customHeight="1" s="34">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>STUDENT INFORMATION</t>
@@ -700,7 +699,7 @@
       </c>
       <c r="C4" s="32" t="inlineStr">
         <is>
-          <t>[Enter your name]</t>
+          <t>Lê Đỗ Hoàng Phúc</t>
         </is>
       </c>
     </row>
@@ -712,7 +711,7 @@
       </c>
       <c r="C5" s="32" t="inlineStr">
         <is>
-          <t>Lê Đỗ Hoàng Phúc</t>
+          <t>QE200057</t>
         </is>
       </c>
     </row>
@@ -724,7 +723,7 @@
       </c>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>QE200057</t>
+          <t>CSD201</t>
         </is>
       </c>
     </row>
@@ -734,20 +733,14 @@
           <t>Assignment:</t>
         </is>
       </c>
-      <c r="C7" s="32" t="inlineStr">
-        <is>
-          <t>CSD201</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Browser History</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18.75" customHeight="1" s="35">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Browser History and Cache Navigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9" ht="18.75" customHeight="1" s="34">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>AI USAGE SUMMARY</t>
@@ -808,7 +801,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="18.75" customHeight="1" s="35">
+    <row r="15" ht="18.75" customHeight="1" s="34">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>AI TOOLS USED</t>
@@ -859,7 +852,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1" s="35">
+    <row r="18" ht="30" customHeight="1" s="34">
       <c r="A18" s="7" t="inlineStr">
         <is>
           <t>Claude</t>
@@ -881,7 +874,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1" s="35">
+    <row r="19" ht="30" customHeight="1" s="34">
       <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Gemini</t>
@@ -903,7 +896,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1" s="35">
+    <row r="20" ht="30" customHeight="1" s="34">
       <c r="A20" s="7" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -926,14 +919,14 @@
       </c>
     </row>
     <row r="21"/>
-    <row r="22" ht="18.75" customHeight="1" s="35">
+    <row r="22" ht="18.75" customHeight="1" s="34">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>CORE PROMPTS DISTRIBUTION BY DTC COMPONENT</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="28.5" customHeight="1" s="35">
+    <row r="23" ht="28.5" customHeight="1" s="34">
       <c r="A23" s="6" t="inlineStr">
         <is>
           <t>DTC Component</t>
@@ -956,8 +949,8 @@
           <t>Decomposition</t>
         </is>
       </c>
-      <c r="B24" s="13" t="n">
-        <v>0</v>
+      <c r="B24" s="14" t="n">
+        <v>1</v>
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
@@ -971,8 +964,8 @@
           <t>Pattern Recognition</t>
         </is>
       </c>
-      <c r="B25" s="13" t="n">
-        <v>0</v>
+      <c r="B25" s="14" t="n">
+        <v>1</v>
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
@@ -986,8 +979,8 @@
           <t>Abstraction</t>
         </is>
       </c>
-      <c r="B26" s="13" t="n">
-        <v>0</v>
+      <c r="B26" s="14" t="n">
+        <v>1</v>
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
@@ -1001,8 +994,8 @@
           <t>Algorithms</t>
         </is>
       </c>
-      <c r="B27" s="13" t="n">
-        <v>0</v>
+      <c r="B27" s="14" t="n">
+        <v>3</v>
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
@@ -1010,6 +1003,19 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
@@ -1027,13 +1033,13 @@
   <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" style="35" min="1" max="1"/>
-    <col width="18" customWidth="1" style="35" min="2" max="3"/>
-    <col width="25" customWidth="1" style="35" min="4" max="4"/>
-    <col width="30" customWidth="1" style="35" min="5" max="5"/>
-    <col width="35" customWidth="1" style="35" min="6" max="6"/>
-    <col width="50" customWidth="1" style="35" min="7" max="7"/>
-    <col width="26.85546875" customWidth="1" style="35" min="8" max="8"/>
+    <col width="8" customWidth="1" style="34" min="1" max="1"/>
+    <col width="18" customWidth="1" style="34" min="2" max="3"/>
+    <col width="25" customWidth="1" style="34" min="4" max="4"/>
+    <col width="30" customWidth="1" style="34" min="5" max="5"/>
+    <col width="35" customWidth="1" style="34" min="6" max="6"/>
+    <col width="50" customWidth="1" style="34" min="7" max="7"/>
+    <col width="26.85546875" customWidth="1" style="34" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1043,14 +1049,14 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1" s="35">
-      <c r="A2" s="34" t="inlineStr">
+    <row r="2" ht="30" customHeight="1" s="34">
+      <c r="A2" s="33" t="inlineStr">
         <is>
           <t>INSTRUCTIONS: Chỉ ghi CORE PROMPTS (Decision/Problem-Solving/Verification). Mỗi entry phải trả lời đầy đủ 4 câu hỏi trong Human Delta.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="39.95" customHeight="1" s="35">
+    <row r="3" ht="39.95" customHeight="1" s="34">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Entry #</t>
@@ -1092,7 +1098,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="99.95" customHeight="1" s="35">
+    <row r="4" ht="99.95" customHeight="1" s="34">
       <c r="A4" s="23" t="inlineStr">
         <is>
           <t>001</t>
@@ -1134,7 +1140,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="99.95" customHeight="1" s="35" thickBot="1">
+    <row r="5" ht="99.95" customHeight="1" s="34" thickBot="1">
       <c r="A5" s="23" t="inlineStr">
         <is>
           <t>002</t>
@@ -1176,7 +1182,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="80.09999999999999" customHeight="1" s="35" thickBot="1">
+    <row r="6" ht="80.09999999999999" customHeight="1" s="34" thickBot="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
           <t>003</t>
@@ -1315,7 +1321,7 @@
       </c>
       <c r="C9" s="24" t="inlineStr">
         <is>
-          <t>Refactoring</t>
+          <t>Algorithms</t>
         </is>
       </c>
       <c r="D9" s="24" t="inlineStr">
@@ -1344,7 +1350,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="10" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A10" s="3" t="n"/>
       <c r="B10" s="3" t="n"/>
       <c r="C10" s="3" t="n"/>
@@ -1354,7 +1360,7 @@
       <c r="G10" s="3" t="n"/>
       <c r="H10" s="3" t="n"/>
     </row>
-    <row r="11" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="11" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A11" s="3" t="n"/>
       <c r="B11" s="3" t="n"/>
       <c r="C11" s="3" t="n"/>
@@ -1364,7 +1370,7 @@
       <c r="G11" s="3" t="n"/>
       <c r="H11" s="3" t="n"/>
     </row>
-    <row r="12" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="12" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A12" s="3" t="n"/>
       <c r="B12" s="3" t="n"/>
       <c r="C12" s="3" t="n"/>
@@ -1374,7 +1380,7 @@
       <c r="G12" s="3" t="n"/>
       <c r="H12" s="3" t="n"/>
     </row>
-    <row r="13" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="13" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A13" s="3" t="n"/>
       <c r="B13" s="3" t="n"/>
       <c r="C13" s="3" t="n"/>
@@ -1384,7 +1390,7 @@
       <c r="G13" s="3" t="n"/>
       <c r="H13" s="3" t="n"/>
     </row>
-    <row r="14" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="14" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A14" s="3" t="n"/>
       <c r="B14" s="3" t="n"/>
       <c r="C14" s="3" t="n"/>
@@ -1394,7 +1400,7 @@
       <c r="G14" s="3" t="n"/>
       <c r="H14" s="3" t="n"/>
     </row>
-    <row r="15" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="15" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A15" s="3" t="n"/>
       <c r="B15" s="3" t="n"/>
       <c r="C15" s="3" t="n"/>
@@ -1404,7 +1410,7 @@
       <c r="G15" s="3" t="n"/>
       <c r="H15" s="3" t="n"/>
     </row>
-    <row r="16" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="16" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A16" s="3" t="n"/>
       <c r="B16" s="3" t="n"/>
       <c r="C16" s="3" t="n"/>
@@ -1414,7 +1420,7 @@
       <c r="G16" s="3" t="n"/>
       <c r="H16" s="3" t="n"/>
     </row>
-    <row r="17" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="17" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A17" s="3" t="n"/>
       <c r="B17" s="3" t="n"/>
       <c r="C17" s="3" t="n"/>
@@ -1424,7 +1430,7 @@
       <c r="G17" s="3" t="n"/>
       <c r="H17" s="3" t="n"/>
     </row>
-    <row r="18" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="18" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A18" s="3" t="n"/>
       <c r="B18" s="3" t="n"/>
       <c r="C18" s="3" t="n"/>
@@ -1434,7 +1440,7 @@
       <c r="G18" s="3" t="n"/>
       <c r="H18" s="3" t="n"/>
     </row>
-    <row r="19" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="19" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A19" s="3" t="n"/>
       <c r="B19" s="3" t="n"/>
       <c r="C19" s="3" t="n"/>
@@ -1444,7 +1450,7 @@
       <c r="G19" s="3" t="n"/>
       <c r="H19" s="3" t="n"/>
     </row>
-    <row r="20" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="20" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A20" s="3" t="n"/>
       <c r="B20" s="3" t="n"/>
       <c r="C20" s="3" t="n"/>
@@ -1454,7 +1460,7 @@
       <c r="G20" s="3" t="n"/>
       <c r="H20" s="3" t="n"/>
     </row>
-    <row r="21" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="21" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A21" s="3" t="n"/>
       <c r="B21" s="3" t="n"/>
       <c r="C21" s="3" t="n"/>
@@ -1464,7 +1470,7 @@
       <c r="G21" s="3" t="n"/>
       <c r="H21" s="3" t="n"/>
     </row>
-    <row r="22" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="22" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A22" s="3" t="n"/>
       <c r="B22" s="3" t="n"/>
       <c r="C22" s="3" t="n"/>
@@ -1474,7 +1480,7 @@
       <c r="G22" s="3" t="n"/>
       <c r="H22" s="3" t="n"/>
     </row>
-    <row r="23" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="23" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A23" s="3" t="n"/>
       <c r="B23" s="3" t="n"/>
       <c r="C23" s="3" t="n"/>
@@ -1484,7 +1490,7 @@
       <c r="G23" s="3" t="n"/>
       <c r="H23" s="3" t="n"/>
     </row>
-    <row r="24" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="24" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A24" s="3" t="n"/>
       <c r="B24" s="3" t="n"/>
       <c r="C24" s="3" t="n"/>
@@ -1494,7 +1500,7 @@
       <c r="G24" s="3" t="n"/>
       <c r="H24" s="3" t="n"/>
     </row>
-    <row r="25" ht="80.09999999999999" customHeight="1" s="35">
+    <row r="25" ht="80.09999999999999" customHeight="1" s="34">
       <c r="A25" s="3" t="n"/>
       <c r="B25" s="3" t="n"/>
       <c r="C25" s="3" t="n"/>
@@ -1523,26 +1529,26 @@
   <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" style="35" min="1" max="1"/>
-    <col width="22" customWidth="1" style="35" min="2" max="2"/>
-    <col width="30" customWidth="1" style="35" min="3" max="6"/>
+    <col width="12" customWidth="1" style="34" min="1" max="1"/>
+    <col width="22" customWidth="1" style="34" min="2" max="2"/>
+    <col width="30" customWidth="1" style="34" min="3" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="37" t="inlineStr">
+      <c r="A1" s="36" t="inlineStr">
         <is>
           <t>HALLUCINATION DETECTION LOG (BẮT BUỘC)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="36" t="inlineStr">
+      <c r="A2" s="35" t="inlineStr">
         <is>
           <t>MỖI PROJECT PHẢI PHÁT HIỆN ÍT NHẤT: Lab (≥1), Assignment (≥2), Project (≥3) cases hallucination</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="39.95" customHeight="1" s="35">
+    <row r="3" ht="39.95" customHeight="1" s="34">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Entry # (from Sheet 2)</t>
@@ -1574,7 +1580,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1" s="35">
+    <row r="4" ht="60" customHeight="1" s="34">
       <c r="A4" s="26" t="inlineStr">
         <is>
           <t>001</t>
@@ -1606,7 +1612,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1" s="35">
+    <row r="5" ht="30" customHeight="1" s="34">
       <c r="A5" s="27" t="inlineStr">
         <is>
           <t>002</t>
@@ -1638,7 +1644,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1" s="35">
+    <row r="6" ht="60" customHeight="1" s="34">
       <c r="A6" s="27" t="inlineStr">
         <is>
           <t>003</t>
@@ -1670,7 +1676,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1" s="35">
+    <row r="7" ht="60" customHeight="1" s="34">
       <c r="A7" s="3" t="n"/>
       <c r="B7" s="3" t="n"/>
       <c r="C7" s="3" t="n"/>
@@ -1678,7 +1684,7 @@
       <c r="E7" s="3" t="n"/>
       <c r="F7" s="3" t="n"/>
     </row>
-    <row r="8" ht="60" customHeight="1" s="35">
+    <row r="8" ht="60" customHeight="1" s="34">
       <c r="A8" s="3" t="n"/>
       <c r="B8" s="3" t="n"/>
       <c r="C8" s="3" t="n"/>
@@ -1686,7 +1692,7 @@
       <c r="E8" s="3" t="n"/>
       <c r="F8" s="3" t="n"/>
     </row>
-    <row r="9" ht="60" customHeight="1" s="35">
+    <row r="9" ht="60" customHeight="1" s="34">
       <c r="A9" s="3" t="n"/>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="3" t="n"/>
@@ -1694,7 +1700,7 @@
       <c r="E9" s="3" t="n"/>
       <c r="F9" s="3" t="n"/>
     </row>
-    <row r="10" ht="60" customHeight="1" s="35">
+    <row r="10" ht="60" customHeight="1" s="34">
       <c r="A10" s="3" t="n"/>
       <c r="B10" s="3" t="n"/>
       <c r="C10" s="3" t="n"/>
@@ -1702,7 +1708,7 @@
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="3" t="n"/>
     </row>
-    <row r="11" ht="60" customHeight="1" s="35">
+    <row r="11" ht="60" customHeight="1" s="34">
       <c r="A11" s="3" t="n"/>
       <c r="B11" s="3" t="n"/>
       <c r="C11" s="3" t="n"/>
@@ -1710,7 +1716,7 @@
       <c r="E11" s="3" t="n"/>
       <c r="F11" s="3" t="n"/>
     </row>
-    <row r="12" ht="60" customHeight="1" s="35">
+    <row r="12" ht="60" customHeight="1" s="34">
       <c r="A12" s="3" t="n"/>
       <c r="B12" s="3" t="n"/>
       <c r="C12" s="3" t="n"/>
@@ -1718,7 +1724,7 @@
       <c r="E12" s="3" t="n"/>
       <c r="F12" s="3" t="n"/>
     </row>
-    <row r="13" ht="60" customHeight="1" s="35">
+    <row r="13" ht="60" customHeight="1" s="34">
       <c r="A13" s="3" t="n"/>
       <c r="B13" s="3" t="n"/>
       <c r="C13" s="3" t="n"/>
@@ -1726,7 +1732,7 @@
       <c r="E13" s="3" t="n"/>
       <c r="F13" s="3" t="n"/>
     </row>
-    <row r="14" ht="60" customHeight="1" s="35">
+    <row r="14" ht="60" customHeight="1" s="34">
       <c r="A14" s="3" t="n"/>
       <c r="B14" s="3" t="n"/>
       <c r="C14" s="3" t="n"/>
@@ -1734,7 +1740,7 @@
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="3" t="n"/>
     </row>
-    <row r="15" ht="60" customHeight="1" s="35">
+    <row r="15" ht="60" customHeight="1" s="34">
       <c r="A15" s="3" t="n"/>
       <c r="B15" s="3" t="n"/>
       <c r="C15" s="3" t="n"/>
@@ -1742,7 +1748,7 @@
       <c r="E15" s="3" t="n"/>
       <c r="F15" s="3" t="n"/>
     </row>
-    <row r="16" ht="60" customHeight="1" s="35">
+    <row r="16" ht="60" customHeight="1" s="34">
       <c r="A16" s="3" t="n"/>
       <c r="B16" s="3" t="n"/>
       <c r="C16" s="3" t="n"/>
@@ -1750,7 +1756,7 @@
       <c r="E16" s="3" t="n"/>
       <c r="F16" s="3" t="n"/>
     </row>
-    <row r="17" ht="60" customHeight="1" s="35">
+    <row r="17" ht="60" customHeight="1" s="34">
       <c r="A17" s="3" t="n"/>
       <c r="B17" s="3" t="n"/>
       <c r="C17" s="3" t="n"/>
@@ -1758,7 +1764,7 @@
       <c r="E17" s="3" t="n"/>
       <c r="F17" s="3" t="n"/>
     </row>
-    <row r="18" ht="60" customHeight="1" s="35">
+    <row r="18" ht="60" customHeight="1" s="34">
       <c r="A18" s="3" t="n"/>
       <c r="B18" s="3" t="n"/>
       <c r="C18" s="3" t="n"/>
@@ -1766,7 +1772,7 @@
       <c r="E18" s="3" t="n"/>
       <c r="F18" s="3" t="n"/>
     </row>
-    <row r="19" ht="60" customHeight="1" s="35">
+    <row r="19" ht="60" customHeight="1" s="34">
       <c r="A19" s="3" t="n"/>
       <c r="B19" s="3" t="n"/>
       <c r="C19" s="3" t="n"/>
@@ -1774,7 +1780,7 @@
       <c r="E19" s="3" t="n"/>
       <c r="F19" s="3" t="n"/>
     </row>
-    <row r="20" ht="60" customHeight="1" s="35">
+    <row r="20" ht="60" customHeight="1" s="34">
       <c r="A20" s="3" t="n"/>
       <c r="B20" s="3" t="n"/>
       <c r="C20" s="3" t="n"/>
@@ -1782,7 +1788,7 @@
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n"/>
     </row>
-    <row r="21" ht="60" customHeight="1" s="35">
+    <row r="21" ht="60" customHeight="1" s="34">
       <c r="A21" s="3" t="n"/>
       <c r="B21" s="3" t="n"/>
       <c r="C21" s="3" t="n"/>
@@ -1790,7 +1796,7 @@
       <c r="E21" s="3" t="n"/>
       <c r="F21" s="3" t="n"/>
     </row>
-    <row r="22" ht="60" customHeight="1" s="35">
+    <row r="22" ht="60" customHeight="1" s="34">
       <c r="A22" s="3" t="n"/>
       <c r="B22" s="3" t="n"/>
       <c r="C22" s="3" t="n"/>
@@ -1798,7 +1804,7 @@
       <c r="E22" s="3" t="n"/>
       <c r="F22" s="3" t="n"/>
     </row>
-    <row r="23" ht="60" customHeight="1" s="35">
+    <row r="23" ht="60" customHeight="1" s="34">
       <c r="A23" s="3" t="n"/>
       <c r="B23" s="3" t="n"/>
       <c r="C23" s="3" t="n"/>
@@ -1806,7 +1812,7 @@
       <c r="E23" s="3" t="n"/>
       <c r="F23" s="3" t="n"/>
     </row>
-    <row r="24" ht="60" customHeight="1" s="35">
+    <row r="24" ht="60" customHeight="1" s="34">
       <c r="A24" s="3" t="n"/>
       <c r="B24" s="3" t="n"/>
       <c r="C24" s="3" t="n"/>
@@ -1814,12 +1820,7 @@
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n"/>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30" ht="18.75" customHeight="1" s="35">
+    <row r="30" ht="18.75" customHeight="1" s="34">
       <c r="A30" s="1" t="inlineStr">
         <is>
           <t>HALLUCINATION TYPES REFERENCE:</t>
@@ -1843,7 +1844,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1" s="35">
+    <row r="32" ht="30" customHeight="1" s="34">
       <c r="A32" s="3" t="inlineStr">
         <is>
           <t>Fabrication</t>
@@ -1860,7 +1861,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="30" customHeight="1" s="35">
+    <row r="33" ht="30" customHeight="1" s="34">
       <c r="A33" s="3" t="inlineStr">
         <is>
           <t>Oversimplification</t>
@@ -1877,7 +1878,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="30" customHeight="1" s="35">
+    <row r="34" ht="30" customHeight="1" s="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
           <t>Logic Error</t>
@@ -1894,7 +1895,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="30" customHeight="1" s="35">
+    <row r="35" ht="30" customHeight="1" s="34">
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t>Outdated Info</t>
@@ -1911,7 +1912,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="45" customHeight="1" s="35">
+    <row r="36" ht="45" customHeight="1" s="34">
       <c r="A36" s="3" t="inlineStr">
         <is>
           <t>Context Misunderstanding</t>
@@ -1950,8 +1951,8 @@
     <col width="60" customWidth="1" style="32" min="2" max="2"/>
     <col width="10" customWidth="1" style="32" min="3" max="3"/>
     <col width="30" customWidth="1" style="32" min="4" max="4"/>
-    <col width="8.7109375" customWidth="1" style="32" min="5" max="7"/>
-    <col width="8.7109375" customWidth="1" style="32" min="8" max="16384"/>
+    <col width="8.7109375" customWidth="1" style="32" min="5" max="8"/>
+    <col width="8.7109375" customWidth="1" style="32" min="9" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1962,14 +1963,13 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="33" t="inlineStr">
+      <c r="A2" s="37" t="inlineStr">
         <is>
           <t>Kiểm tra kỹ trước khi nộp. MỖI ENTRY phải pass ≥4/5 tiêu chí dưới đây.</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4" ht="18.75" customHeight="1" s="35">
+    <row r="4" ht="18.75" customHeight="1" s="34">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>A. KIỂM TRA CHẤT LƯỢNG MỖI ENTRY (Pass ≥4/5)</t>
@@ -2088,8 +2088,7 @@
       </c>
       <c r="D10" s="17" t="n"/>
     </row>
-    <row r="11"/>
-    <row r="12" ht="18.75" customHeight="1" s="35">
+    <row r="12" ht="18.75" customHeight="1" s="34">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>B. KIỂM TRA TỔNG THỂ LOG</t>
@@ -2208,8 +2207,7 @@
       </c>
       <c r="D18" s="17" t="n"/>
     </row>
-    <row r="19"/>
-    <row r="20" ht="15.75" customHeight="1" s="35">
+    <row r="20" ht="15.75" customHeight="1" s="34">
       <c r="A20" s="18" t="inlineStr">
         <is>
           <t>⚠️ LƯU Ý QUAN TRỌNG:</t>
@@ -2230,9 +2228,7 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25" ht="18.75" customHeight="1" s="35">
+    <row r="25" ht="18.75" customHeight="1" s="34">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>C. CHUẨN BỊ CHO ORAL VIVAS (Q&amp;A)</t>
@@ -2246,7 +2242,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="57" customHeight="1" s="35">
+    <row r="27" ht="57" customHeight="1" s="34">
       <c r="A27" s="21" t="inlineStr">
         <is>
           <t>Entry #</t>
@@ -2268,7 +2264,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="120" customHeight="1" s="35">
+    <row r="28" ht="120" customHeight="1" s="34">
       <c r="A28" s="23" t="inlineStr">
         <is>
           <t>002</t>
@@ -2290,7 +2286,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="75" customHeight="1" s="35">
+    <row r="29" ht="75" customHeight="1" s="34">
       <c r="A29" s="23" t="inlineStr">
         <is>
           <t>004</t>
@@ -2312,7 +2308,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="90" customHeight="1" s="35">
+    <row r="30" ht="90" customHeight="1" s="34">
       <c r="A30" s="23" t="inlineStr">
         <is>
           <t>006</t>

</xml_diff>